<commit_message>
Inclui relatórios 028-036 (PDF 422-430) na relação do databook
Acrescenta colunas de arquivo PDF e página no PDF de origem.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YBR97vd31m3ywVeV1zohhZ
</commit_message>
<xml_diff>
--- a/saida/Relacao_Databook_395-421.xlsx
+++ b/saida/Relacao_Databook_395-421.xlsx
@@ -11,8 +11,8 @@
     <sheet name="Resumo por relatório" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Relação por spool'!$A$1:$J$44</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Resumo por relatório'!$A$1:$J$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Relação por spool'!$A$1:$K$70</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Resumo por relatório'!$A$1:$K$37</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J44"/>
+  <dimension ref="A1:K70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -471,8 +471,9 @@
     <col width="9" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="70" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="70" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -518,10 +519,15 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Página no databook</t>
+          <t>Arquivo PDF</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Página no PDF</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Observação</t>
         </is>
@@ -564,10 +570,15 @@
           <t>Aprovado</t>
         </is>
       </c>
-      <c r="I2" s="2" t="n">
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>395-421.pdf</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="J2" s="4" t="inlineStr">
+      <c r="K2" s="4" t="inlineStr">
         <is>
           <t>Croqui: Divisão entre spools na junta 8; juntas 4 e 15 solda de campo; spool 02 com sobremetal</t>
         </is>
@@ -610,10 +621,15 @@
           <t>Aprovado</t>
         </is>
       </c>
-      <c r="I3" s="2" t="n">
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>395-421.pdf</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="J3" s="4" t="inlineStr">
+      <c r="K3" s="4" t="inlineStr">
         <is>
           <t>Croqui: Divisão entre spools na junta 8; juntas 4 e 15 solda de campo; spool 02 com sobremetal</t>
         </is>
@@ -656,10 +672,15 @@
           <t>Aprovado</t>
         </is>
       </c>
-      <c r="I4" s="2" t="n">
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>395-421.pdf</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="J4" s="4" t="inlineStr">
+      <c r="K4" s="4" t="inlineStr">
         <is>
           <t>Croqui: Spools divididos nas juntas 13, 11 e 09</t>
         </is>
@@ -702,10 +723,15 @@
           <t>Aprovado</t>
         </is>
       </c>
-      <c r="I5" s="2" t="n">
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>395-421.pdf</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="J5" s="4" t="inlineStr">
+      <c r="K5" s="4" t="inlineStr">
         <is>
           <t>Croqui: Spools divididos nas juntas 13, 11 e 09</t>
         </is>
@@ -748,10 +774,15 @@
           <t>Aprovado</t>
         </is>
       </c>
-      <c r="I6" s="2" t="n">
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>395-421.pdf</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="J6" s="4" t="inlineStr">
+      <c r="K6" s="4" t="inlineStr">
         <is>
           <t>Croqui: Spools divididos nas juntas 13, 11 e 09</t>
         </is>
@@ -794,10 +825,15 @@
           <t>Aprovado</t>
         </is>
       </c>
-      <c r="I7" s="2" t="n">
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>395-421.pdf</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="J7" s="4" t="inlineStr">
+      <c r="K7" s="4" t="inlineStr">
         <is>
           <t>Croqui: Spools divididos nas juntas 13, 11 e 09</t>
         </is>
@@ -836,10 +872,15 @@
           <t>Aprovado</t>
         </is>
       </c>
-      <c r="I8" s="2" t="n">
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>395-421.pdf</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="J8" s="4" t="inlineStr">
+      <c r="K8" s="4" t="inlineStr">
         <is>
           <t>TAG não consta no relatório (referência é o isométrico)</t>
         </is>
@@ -882,10 +923,15 @@
           <t>Aprovado</t>
         </is>
       </c>
-      <c r="I9" s="2" t="n">
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>395-421.pdf</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="J9" s="4" t="inlineStr">
+      <c r="K9" s="4" t="inlineStr">
         <is>
           <t>Prefixo de módulo MO7 removido; Spool não identificado no croqui – considerado spool único 001</t>
         </is>
@@ -928,10 +974,15 @@
           <t>Aprovado</t>
         </is>
       </c>
-      <c r="I10" s="2" t="n">
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>395-421.pdf</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="J10" s="4" t="inlineStr">
+      <c r="K10" s="4" t="inlineStr">
         <is>
           <t>Croqui: Extremidades com sobremetal</t>
         </is>
@@ -974,10 +1025,15 @@
           <t>Aprovado</t>
         </is>
       </c>
-      <c r="I11" s="2" t="n">
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>395-421.pdf</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="J11" s="4" t="inlineStr">
+      <c r="K11" s="4" t="inlineStr">
         <is>
           <t>Croqui: Spool dividido na junta 19; extremidade 01 com sobremetal</t>
         </is>
@@ -1020,10 +1076,15 @@
           <t>Aprovado</t>
         </is>
       </c>
-      <c r="I12" s="2" t="n">
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>395-421.pdf</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="J12" s="4" t="inlineStr">
+      <c r="K12" s="4" t="inlineStr">
         <is>
           <t>Croqui: Spool dividido na junta 19; extremidade 01 com sobremetal</t>
         </is>
@@ -1066,10 +1127,15 @@
           <t>Aprovado</t>
         </is>
       </c>
-      <c r="I13" s="2" t="n">
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>395-421.pdf</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="J13" s="4" t="inlineStr">
+      <c r="K13" s="4" t="inlineStr">
         <is>
           <t>Spool não identificado no croqui – considerado spool único 001; Croqui: Extremidade com sobremetal</t>
         </is>
@@ -1112,10 +1178,15 @@
           <t>Aprovado</t>
         </is>
       </c>
-      <c r="I14" s="2" t="n">
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>395-421.pdf</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="J14" s="4" t="inlineStr">
+      <c r="K14" s="4" t="inlineStr">
         <is>
           <t>Spool não identificado no croqui – considerado spool único 001</t>
         </is>
@@ -1158,10 +1229,15 @@
           <t>Aprovado</t>
         </is>
       </c>
-      <c r="I15" s="2" t="n">
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>395-421.pdf</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="J15" s="4" t="inlineStr">
+      <c r="K15" s="4" t="inlineStr">
         <is>
           <t>Croqui: Spool dividido na junta 4</t>
         </is>
@@ -1204,10 +1280,15 @@
           <t>Aprovado</t>
         </is>
       </c>
-      <c r="I16" s="2" t="n">
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>395-421.pdf</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="J16" s="4" t="inlineStr">
+      <c r="K16" s="4" t="inlineStr">
         <is>
           <t>Croqui: Spool dividido na junta 4</t>
         </is>
@@ -1246,10 +1327,15 @@
           <t>Aprovado</t>
         </is>
       </c>
-      <c r="I17" s="2" t="n">
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>395-421.pdf</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="J17" s="4" t="inlineStr">
+      <c r="K17" s="4" t="inlineStr">
         <is>
           <t>TAG não consta no relatório (referência é o isométrico)</t>
         </is>
@@ -1292,10 +1378,15 @@
           <t>Aprovado</t>
         </is>
       </c>
-      <c r="I18" s="2" t="n">
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>395-421.pdf</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="J18" s="4" t="inlineStr">
+      <c r="K18" s="4" t="inlineStr">
         <is>
           <t>Croqui: Spool dividido na junta 8</t>
         </is>
@@ -1338,10 +1429,15 @@
           <t>Aprovado</t>
         </is>
       </c>
-      <c r="I19" s="2" t="n">
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>395-421.pdf</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="J19" s="4" t="inlineStr">
+      <c r="K19" s="4" t="inlineStr">
         <is>
           <t>Croqui: Spool dividido na junta 8</t>
         </is>
@@ -1384,10 +1480,15 @@
           <t>Aprovado</t>
         </is>
       </c>
-      <c r="I20" s="2" t="n">
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>395-421.pdf</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="J20" s="4" t="inlineStr">
+      <c r="K20" s="4" t="inlineStr">
         <is>
           <t>Prefixo de módulo MO8 removido; Spool não identificado no croqui – considerado spool único 001</t>
         </is>
@@ -1430,10 +1531,15 @@
           <t>Aprovado</t>
         </is>
       </c>
-      <c r="I21" s="2" t="n">
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>395-421.pdf</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="J21" s="4" t="inlineStr">
+      <c r="K21" s="4" t="inlineStr">
         <is>
           <t>Prefixo de módulo MO5 removido; Spool não identificado no croqui – considerado spool único 001</t>
         </is>
@@ -1472,10 +1578,15 @@
           <t>Aprovado</t>
         </is>
       </c>
-      <c r="I22" s="2" t="n">
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>395-421.pdf</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="J22" s="4" t="inlineStr">
+      <c r="K22" s="4" t="inlineStr">
         <is>
           <t>TAG não consta no relatório (referência é o isométrico); Spool não identificado no croqui – considerado spool único 001; Croqui: Extremidades FT (solda de campo)</t>
         </is>
@@ -1514,10 +1625,15 @@
           <t>Aprovado</t>
         </is>
       </c>
-      <c r="I23" s="2" t="n">
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>395-421.pdf</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="J23" s="4" t="inlineStr">
+      <c r="K23" s="4" t="inlineStr">
         <is>
           <t>TAG não consta no relatório (referência é o isométrico); Spool não identificado no croqui – considerado spool único 001; Croqui: Extremidade FT (solda de campo)</t>
         </is>
@@ -1556,10 +1672,15 @@
           <t>Aprovado</t>
         </is>
       </c>
-      <c r="I24" s="2" t="n">
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>395-421.pdf</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="n">
         <v>16</v>
       </c>
-      <c r="J24" s="4" t="inlineStr">
+      <c r="K24" s="4" t="inlineStr">
         <is>
           <t>TAG não consta no relatório (referência é o isométrico); Spool não identificado no croqui – considerado spool único 001; Croqui idêntico ao do relatório 007; Croqui: Extremidade com sobremetal</t>
         </is>
@@ -1598,10 +1719,15 @@
           <t>Aprovado</t>
         </is>
       </c>
-      <c r="I25" s="2" t="n">
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>395-421.pdf</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="J25" s="4" t="inlineStr">
+      <c r="K25" s="4" t="inlineStr">
         <is>
           <t>TAG não consta no relatório (referência é o isométrico); Croqui idêntico ao do relatório 005; Croqui: Extremidades com sobremetal</t>
         </is>
@@ -1640,10 +1766,15 @@
           <t>Aprovado</t>
         </is>
       </c>
-      <c r="I26" s="2" t="n">
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>395-421.pdf</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="J26" s="4" t="inlineStr">
+      <c r="K26" s="4" t="inlineStr">
         <is>
           <t>TAG não consta no relatório (referência é o isométrico)</t>
         </is>
@@ -1682,10 +1813,15 @@
           <t>Aprovado</t>
         </is>
       </c>
-      <c r="I27" s="2" t="n">
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>395-421.pdf</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="n">
         <v>19</v>
       </c>
-      <c r="J27" s="4" t="inlineStr">
+      <c r="K27" s="4" t="inlineStr">
         <is>
           <t>TAG não consta no relatório (referência é o isométrico); Spool não identificado no croqui – considerado spool único 001; Croqui idêntico ao do relatório 008</t>
         </is>
@@ -1724,10 +1860,15 @@
           <t>Aprovado</t>
         </is>
       </c>
-      <c r="I28" s="2" t="n">
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>395-421.pdf</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="J28" s="4" t="inlineStr">
+      <c r="K28" s="4" t="inlineStr">
         <is>
           <t>TAG não consta no relatório (referência é o isométrico); Croqui idêntico ao do relatório 009; Croqui: Spool dividido na junta 4</t>
         </is>
@@ -1766,10 +1907,15 @@
           <t>Aprovado</t>
         </is>
       </c>
-      <c r="I29" s="2" t="n">
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>395-421.pdf</t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="J29" s="4" t="inlineStr">
+      <c r="K29" s="4" t="inlineStr">
         <is>
           <t>TAG não consta no relatório (referência é o isométrico); Croqui idêntico ao do relatório 009; Croqui: Spool dividido na junta 4</t>
         </is>
@@ -1808,12 +1954,17 @@
           <t>Aprovado</t>
         </is>
       </c>
-      <c r="I30" s="2" t="n">
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>395-421.pdf</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="n">
         <v>21</v>
       </c>
-      <c r="J30" s="4" t="inlineStr">
-        <is>
-          <t>TAG não consta no relatório (referência é o isométrico); Croqui idêntico ao do relatório 002; Croqui: Spools divididos nas juntas 13, 11 e 09</t>
+      <c r="K30" s="4" t="inlineStr">
+        <is>
+          <t>Mesmo desenho dos relatórios 036; TAG não consta no relatório (referência é o isométrico); Croqui idêntico ao do relatório 002; Croqui: Spools divididos nas juntas 13, 11 e 09</t>
         </is>
       </c>
     </row>
@@ -1850,12 +2001,17 @@
           <t>Aprovado</t>
         </is>
       </c>
-      <c r="I31" s="2" t="n">
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>395-421.pdf</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="n">
         <v>21</v>
       </c>
-      <c r="J31" s="4" t="inlineStr">
-        <is>
-          <t>TAG não consta no relatório (referência é o isométrico); Croqui idêntico ao do relatório 002; Croqui: Spools divididos nas juntas 13, 11 e 09</t>
+      <c r="K31" s="4" t="inlineStr">
+        <is>
+          <t>Mesmo desenho dos relatórios 036; TAG não consta no relatório (referência é o isométrico); Croqui idêntico ao do relatório 002; Croqui: Spools divididos nas juntas 13, 11 e 09</t>
         </is>
       </c>
     </row>
@@ -1892,12 +2048,17 @@
           <t>Aprovado</t>
         </is>
       </c>
-      <c r="I32" s="2" t="n">
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>395-421.pdf</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="n">
         <v>21</v>
       </c>
-      <c r="J32" s="4" t="inlineStr">
-        <is>
-          <t>TAG não consta no relatório (referência é o isométrico); Croqui idêntico ao do relatório 002; Croqui: Spools divididos nas juntas 13, 11 e 09</t>
+      <c r="K32" s="4" t="inlineStr">
+        <is>
+          <t>Mesmo desenho dos relatórios 036; TAG não consta no relatório (referência é o isométrico); Croqui idêntico ao do relatório 002; Croqui: Spools divididos nas juntas 13, 11 e 09</t>
         </is>
       </c>
     </row>
@@ -1934,12 +2095,17 @@
           <t>Aprovado</t>
         </is>
       </c>
-      <c r="I33" s="2" t="n">
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>395-421.pdf</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="n">
         <v>21</v>
       </c>
-      <c r="J33" s="4" t="inlineStr">
-        <is>
-          <t>TAG não consta no relatório (referência é o isométrico); Croqui idêntico ao do relatório 002; Croqui: Spools divididos nas juntas 13, 11 e 09</t>
+      <c r="K33" s="4" t="inlineStr">
+        <is>
+          <t>Mesmo desenho dos relatórios 036; TAG não consta no relatório (referência é o isométrico); Croqui idêntico ao do relatório 002; Croqui: Spools divididos nas juntas 13, 11 e 09</t>
         </is>
       </c>
     </row>
@@ -1980,10 +2146,15 @@
           <t>Aprovado</t>
         </is>
       </c>
-      <c r="I34" s="2" t="n">
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>395-421.pdf</t>
+        </is>
+      </c>
+      <c r="J34" s="2" t="n">
         <v>22</v>
       </c>
-      <c r="J34" s="4" t="inlineStr">
+      <c r="K34" s="4" t="inlineStr">
         <is>
           <t>Prefixo de módulo MO7 removido; Spool não identificado no croqui – considerado spool único 001</t>
         </is>
@@ -2026,10 +2197,15 @@
           <t>Aprovado</t>
         </is>
       </c>
-      <c r="I35" s="2" t="n">
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t>395-421.pdf</t>
+        </is>
+      </c>
+      <c r="J35" s="2" t="n">
         <v>23</v>
       </c>
-      <c r="J35" s="4" t="inlineStr">
+      <c r="K35" s="4" t="inlineStr">
         <is>
           <t>Prefixo de módulo MO6 removido</t>
         </is>
@@ -2072,10 +2248,15 @@
           <t>Aprovado</t>
         </is>
       </c>
-      <c r="I36" s="2" t="n">
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>395-421.pdf</t>
+        </is>
+      </c>
+      <c r="J36" s="2" t="n">
         <v>24</v>
       </c>
-      <c r="J36" s="4" t="inlineStr">
+      <c r="K36" s="4" t="inlineStr">
         <is>
           <t>Prefixo de módulo MO7 removido; Croqui: Spool dividido nas juntas 06 e 20</t>
         </is>
@@ -2118,10 +2299,15 @@
           <t>Aprovado</t>
         </is>
       </c>
-      <c r="I37" s="2" t="n">
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>395-421.pdf</t>
+        </is>
+      </c>
+      <c r="J37" s="2" t="n">
         <v>24</v>
       </c>
-      <c r="J37" s="4" t="inlineStr">
+      <c r="K37" s="4" t="inlineStr">
         <is>
           <t>Prefixo de módulo MO7 removido; Croqui: Spool dividido nas juntas 06 e 20</t>
         </is>
@@ -2164,10 +2350,15 @@
           <t>Aprovado</t>
         </is>
       </c>
-      <c r="I38" s="2" t="n">
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>395-421.pdf</t>
+        </is>
+      </c>
+      <c r="J38" s="2" t="n">
         <v>24</v>
       </c>
-      <c r="J38" s="4" t="inlineStr">
+      <c r="K38" s="4" t="inlineStr">
         <is>
           <t>Prefixo de módulo MO7 removido; Croqui: Spool dividido nas juntas 06 e 20</t>
         </is>
@@ -2210,10 +2401,15 @@
           <t>Aprovado</t>
         </is>
       </c>
-      <c r="I39" s="2" t="n">
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>395-421.pdf</t>
+        </is>
+      </c>
+      <c r="J39" s="2" t="n">
         <v>25</v>
       </c>
-      <c r="J39" s="4" t="inlineStr">
+      <c r="K39" s="4" t="inlineStr">
         <is>
           <t>Prefixo de módulo MO5 removido</t>
         </is>
@@ -2256,10 +2452,15 @@
           <t>Aprovado</t>
         </is>
       </c>
-      <c r="I40" s="2" t="n">
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>395-421.pdf</t>
+        </is>
+      </c>
+      <c r="J40" s="2" t="n">
         <v>26</v>
       </c>
-      <c r="J40" s="4" t="inlineStr">
+      <c r="K40" s="4" t="inlineStr">
         <is>
           <t>Prefixo de módulo MO8 removido; Croqui: Spool dividido nas juntas 04 e 12</t>
         </is>
@@ -2302,10 +2503,15 @@
           <t>Aprovado</t>
         </is>
       </c>
-      <c r="I41" s="2" t="n">
+      <c r="I41" s="2" t="inlineStr">
+        <is>
+          <t>395-421.pdf</t>
+        </is>
+      </c>
+      <c r="J41" s="2" t="n">
         <v>26</v>
       </c>
-      <c r="J41" s="4" t="inlineStr">
+      <c r="K41" s="4" t="inlineStr">
         <is>
           <t>Prefixo de módulo MO8 removido; Croqui: Spool dividido nas juntas 04 e 12</t>
         </is>
@@ -2348,10 +2554,15 @@
           <t>Aprovado</t>
         </is>
       </c>
-      <c r="I42" s="2" t="n">
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>395-421.pdf</t>
+        </is>
+      </c>
+      <c r="J42" s="2" t="n">
         <v>26</v>
       </c>
-      <c r="J42" s="4" t="inlineStr">
+      <c r="K42" s="4" t="inlineStr">
         <is>
           <t>Prefixo de módulo MO8 removido; Croqui: Spool dividido nas juntas 04 e 12</t>
         </is>
@@ -2394,10 +2605,15 @@
           <t>Aprovado</t>
         </is>
       </c>
-      <c r="I43" s="2" t="n">
+      <c r="I43" s="2" t="inlineStr">
+        <is>
+          <t>395-421.pdf</t>
+        </is>
+      </c>
+      <c r="J43" s="2" t="n">
         <v>27</v>
       </c>
-      <c r="J43" s="4" t="inlineStr">
+      <c r="K43" s="4" t="inlineStr">
         <is>
           <t>Prefixo de módulo MO5 removido; Croqui: Spool dividido na junta 04</t>
         </is>
@@ -2440,17 +2656,1268 @@
           <t>Aprovado</t>
         </is>
       </c>
-      <c r="I44" s="2" t="n">
+      <c r="I44" s="2" t="inlineStr">
+        <is>
+          <t>395-421.pdf</t>
+        </is>
+      </c>
+      <c r="J44" s="2" t="n">
         <v>27</v>
       </c>
-      <c r="J44" s="4" t="inlineStr">
+      <c r="K44" s="4" t="inlineStr">
         <is>
           <t>Prefixo de módulo MO5 removido; Croqui: Spool dividido na junta 04</t>
         </is>
       </c>
     </row>
+    <row r="45">
+      <c r="A45" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>028</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>Relatório Dimensional</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="n">
+        <v>46265</v>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>I-IS-025-421-510-46-9067</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr"/>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="I45" s="2" t="inlineStr">
+        <is>
+          <t>422-430.pdf</t>
+        </is>
+      </c>
+      <c r="J45" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K45" s="4" t="inlineStr">
+        <is>
+          <t>TAG não consta no relatório (referência é o isométrico); Croqui: Spools divididos nas juntas 04 e 05; extremidades FT</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>028</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>Relatório Dimensional</t>
+        </is>
+      </c>
+      <c r="D46" s="3" t="n">
+        <v>46265</v>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>I-IS-025-421-510-46-9067</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>002</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr"/>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="I46" s="2" t="inlineStr">
+        <is>
+          <t>422-430.pdf</t>
+        </is>
+      </c>
+      <c r="J46" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K46" s="4" t="inlineStr">
+        <is>
+          <t>TAG não consta no relatório (referência é o isométrico); Croqui: Spools divididos nas juntas 04 e 05; extremidades FT</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>028</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>Relatório Dimensional</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="n">
+        <v>46265</v>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>I-IS-025-421-510-46-9067</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>003</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr"/>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="I47" s="2" t="inlineStr">
+        <is>
+          <t>422-430.pdf</t>
+        </is>
+      </c>
+      <c r="J47" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K47" s="4" t="inlineStr">
+        <is>
+          <t>TAG não consta no relatório (referência é o isométrico); Croqui: Spools divididos nas juntas 04 e 05; extremidades FT</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>029</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>Relatório Dimensional</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="n">
+        <v>46260</v>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>I-IS-025-421-510-46-9141</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr"/>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="I48" s="2" t="inlineStr">
+        <is>
+          <t>422-430.pdf</t>
+        </is>
+      </c>
+      <c r="J48" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K48" s="4" t="inlineStr">
+        <is>
+          <t>TAG não consta no relatório (referência é o isométrico); Croqui idêntico ao do relatório 006; Croqui: Spool dividido na junta 19; extremidade 01 com sobremetal</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>029</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>Relatório Dimensional</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="n">
+        <v>46260</v>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>I-IS-025-421-510-46-9141</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>002</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="inlineStr"/>
+      <c r="H49" s="2" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="I49" s="2" t="inlineStr">
+        <is>
+          <t>422-430.pdf</t>
+        </is>
+      </c>
+      <c r="J49" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K49" s="4" t="inlineStr">
+        <is>
+          <t>TAG não consta no relatório (referência é o isométrico); Croqui idêntico ao do relatório 006; Croqui: Spool dividido na junta 19; extremidade 01 com sobremetal</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>030</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>Relatório Dimensional</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="n">
+        <v>46266</v>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>MO8-6´´-B3B-MR-5407B-PP-2 FL 2/2</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>6"-B3B-MR-5407B</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="I50" s="2" t="inlineStr">
+        <is>
+          <t>422-430.pdf</t>
+        </is>
+      </c>
+      <c r="J50" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="K50" s="4" t="inlineStr">
+        <is>
+          <t>Prefixo de módulo MO8 removido; Croqui: Spool dividido nas juntas 08, 16 e 28</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>030</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>Relatório Dimensional</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="n">
+        <v>46266</v>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>MO8-6´´-B3B-MR-5407B-PP-2 FL 2/2</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>002</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>6"-B3B-MR-5407B</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="I51" s="2" t="inlineStr">
+        <is>
+          <t>422-430.pdf</t>
+        </is>
+      </c>
+      <c r="J51" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="K51" s="4" t="inlineStr">
+        <is>
+          <t>Prefixo de módulo MO8 removido; Croqui: Spool dividido nas juntas 08, 16 e 28</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>030</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>Relatório Dimensional</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="n">
+        <v>46266</v>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>MO8-6´´-B3B-MR-5407B-PP-2 FL 2/2</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>003</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>6"-B3B-MR-5407B</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="I52" s="2" t="inlineStr">
+        <is>
+          <t>422-430.pdf</t>
+        </is>
+      </c>
+      <c r="J52" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="K52" s="4" t="inlineStr">
+        <is>
+          <t>Prefixo de módulo MO8 removido; Croqui: Spool dividido nas juntas 08, 16 e 28</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>030</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>Relatório Dimensional</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="n">
+        <v>46266</v>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>MO8-6´´-B3B-MR-5407B-PP-2 FL 2/2</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>004</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t>6"-B3B-MR-5407B</t>
+        </is>
+      </c>
+      <c r="H53" s="2" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="I53" s="2" t="inlineStr">
+        <is>
+          <t>422-430.pdf</t>
+        </is>
+      </c>
+      <c r="J53" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="K53" s="4" t="inlineStr">
+        <is>
+          <t>Prefixo de módulo MO8 removido; Croqui: Spool dividido nas juntas 08, 16 e 28</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>031</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>Relatório Dimensional</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="n">
+        <v>46265</v>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>I-IS-025-421-510-46-9048</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr"/>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="I54" s="2" t="inlineStr">
+        <is>
+          <t>422-430.pdf</t>
+        </is>
+      </c>
+      <c r="J54" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="K54" s="4" t="inlineStr">
+        <is>
+          <t>TAG não consta no relatório (referência é o isométrico); Croqui: Spools divididos nas juntas 08 e 09; extremidades FT</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>031</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>Relatório Dimensional</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="n">
+        <v>46265</v>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>I-IS-025-421-510-46-9048</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>002</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="inlineStr"/>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="I55" s="2" t="inlineStr">
+        <is>
+          <t>422-430.pdf</t>
+        </is>
+      </c>
+      <c r="J55" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="K55" s="4" t="inlineStr">
+        <is>
+          <t>TAG não consta no relatório (referência é o isométrico); Croqui: Spools divididos nas juntas 08 e 09; extremidades FT</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>031</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>Relatório Dimensional</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="n">
+        <v>46265</v>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>I-IS-025-421-510-46-9048</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>003</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr"/>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="I56" s="2" t="inlineStr">
+        <is>
+          <t>422-430.pdf</t>
+        </is>
+      </c>
+      <c r="J56" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="K56" s="4" t="inlineStr">
+        <is>
+          <t>TAG não consta no relatório (referência é o isométrico); Croqui: Spools divididos nas juntas 08 e 09; extremidades FT</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>032</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>Relatório Dimensional</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="n">
+        <v>46265</v>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>I-IS-025-421-510-46-9049</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="inlineStr"/>
+      <c r="H57" s="2" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="I57" s="2" t="inlineStr">
+        <is>
+          <t>422-430.pdf</t>
+        </is>
+      </c>
+      <c r="J57" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="K57" s="4" t="inlineStr">
+        <is>
+          <t>TAG não consta no relatório (referência é o isométrico); Croqui: Spools divididos nas juntas 24 e 25; extremidades FT</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>032</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>Relatório Dimensional</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="n">
+        <v>46265</v>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>I-IS-025-421-510-46-9049</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>002</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr"/>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="I58" s="2" t="inlineStr">
+        <is>
+          <t>422-430.pdf</t>
+        </is>
+      </c>
+      <c r="J58" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="K58" s="4" t="inlineStr">
+        <is>
+          <t>TAG não consta no relatório (referência é o isométrico); Croqui: Spools divididos nas juntas 24 e 25; extremidades FT</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>032</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>Relatório Dimensional</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="n">
+        <v>46265</v>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>I-IS-025-421-510-46-9049</t>
+        </is>
+      </c>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>003</t>
+        </is>
+      </c>
+      <c r="G59" s="2" t="inlineStr"/>
+      <c r="H59" s="2" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="I59" s="2" t="inlineStr">
+        <is>
+          <t>422-430.pdf</t>
+        </is>
+      </c>
+      <c r="J59" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="K59" s="4" t="inlineStr">
+        <is>
+          <t>TAG não consta no relatório (referência é o isométrico); Croqui: Spools divididos nas juntas 24 e 25; extremidades FT</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="n">
+        <v>59</v>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>033</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>Relatório Dimensional</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="n">
+        <v>46266</v>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>6´´-B3B-MR-5407A-PP-2</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>002</t>
+        </is>
+      </c>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>6"-B3B-MR-5407A</t>
+        </is>
+      </c>
+      <c r="H60" s="2" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="I60" s="2" t="inlineStr">
+        <is>
+          <t>422-430.pdf</t>
+        </is>
+      </c>
+      <c r="J60" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="K60" s="4" t="inlineStr">
+        <is>
+          <t>Croqui: Spool dividido nas juntas 08 e 12</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>033</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>Relatório Dimensional</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="n">
+        <v>46266</v>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>6´´-B3B-MR-5407A-PP-2</t>
+        </is>
+      </c>
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>003</t>
+        </is>
+      </c>
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>6"-B3B-MR-5407A</t>
+        </is>
+      </c>
+      <c r="H61" s="2" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="I61" s="2" t="inlineStr">
+        <is>
+          <t>422-430.pdf</t>
+        </is>
+      </c>
+      <c r="J61" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="K61" s="4" t="inlineStr">
+        <is>
+          <t>Croqui: Spool dividido nas juntas 08 e 12</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="n">
+        <v>61</v>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>034</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>Relatório Dimensional</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="n">
+        <v>46259</v>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>I-IS-025-421-510-46-9137</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="inlineStr"/>
+      <c r="H62" s="2" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="I62" s="2" t="inlineStr">
+        <is>
+          <t>422-430.pdf</t>
+        </is>
+      </c>
+      <c r="J62" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="K62" s="4" t="inlineStr">
+        <is>
+          <t>TAG não consta no relatório (referência é o isométrico); Croqui idêntico ao do relatório 001; Croqui: Spool dividido na junta 8; juntas 4 e 15 FW</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="n">
+        <v>62</v>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>034</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>Relatório Dimensional</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="n">
+        <v>46259</v>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>I-IS-025-421-510-46-9137</t>
+        </is>
+      </c>
+      <c r="F63" s="2" t="inlineStr">
+        <is>
+          <t>002</t>
+        </is>
+      </c>
+      <c r="G63" s="2" t="inlineStr"/>
+      <c r="H63" s="2" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="I63" s="2" t="inlineStr">
+        <is>
+          <t>422-430.pdf</t>
+        </is>
+      </c>
+      <c r="J63" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="K63" s="4" t="inlineStr">
+        <is>
+          <t>TAG não consta no relatório (referência é o isométrico); Croqui idêntico ao do relatório 001; Croqui: Spool dividido na junta 8; juntas 4 e 15 FW</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="n">
+        <v>63</v>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>035</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>Relatório Dimensional</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="n">
+        <v>46265</v>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>I-IS-025-421-510-46-9066</t>
+        </is>
+      </c>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="G64" s="2" t="inlineStr"/>
+      <c r="H64" s="2" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="I64" s="2" t="inlineStr">
+        <is>
+          <t>422-430.pdf</t>
+        </is>
+      </c>
+      <c r="J64" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="K64" s="4" t="inlineStr">
+        <is>
+          <t>TAG não consta no relatório (referência é o isométrico); Croqui: Spools divididos nas juntas 16 e 17; extremidades FT</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="n">
+        <v>64</v>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>035</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>Relatório Dimensional</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="n">
+        <v>46265</v>
+      </c>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>I-IS-025-421-510-46-9066</t>
+        </is>
+      </c>
+      <c r="F65" s="2" t="inlineStr">
+        <is>
+          <t>002</t>
+        </is>
+      </c>
+      <c r="G65" s="2" t="inlineStr"/>
+      <c r="H65" s="2" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="I65" s="2" t="inlineStr">
+        <is>
+          <t>422-430.pdf</t>
+        </is>
+      </c>
+      <c r="J65" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="K65" s="4" t="inlineStr">
+        <is>
+          <t>TAG não consta no relatório (referência é o isométrico); Croqui: Spools divididos nas juntas 16 e 17; extremidades FT</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="n">
+        <v>65</v>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>035</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>Relatório Dimensional</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="n">
+        <v>46265</v>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>I-IS-025-421-510-46-9066</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>003</t>
+        </is>
+      </c>
+      <c r="G66" s="2" t="inlineStr"/>
+      <c r="H66" s="2" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="I66" s="2" t="inlineStr">
+        <is>
+          <t>422-430.pdf</t>
+        </is>
+      </c>
+      <c r="J66" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="K66" s="4" t="inlineStr">
+        <is>
+          <t>TAG não consta no relatório (referência é o isométrico); Croqui: Spools divididos nas juntas 16 e 17; extremidades FT</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="n">
+        <v>66</v>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>036</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>Relatório Dimensional</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="n">
+        <v>46259</v>
+      </c>
+      <c r="E67" s="2" t="inlineStr">
+        <is>
+          <t>I-IS-025-421-510-46-9138</t>
+        </is>
+      </c>
+      <c r="F67" s="2" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="G67" s="2" t="inlineStr"/>
+      <c r="H67" s="2" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="I67" s="2" t="inlineStr">
+        <is>
+          <t>422-430.pdf</t>
+        </is>
+      </c>
+      <c r="J67" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="K67" s="4" t="inlineStr">
+        <is>
+          <t>Mesmo desenho dos relatórios 021; TAG não consta no relatório (referência é o isométrico); Croqui idêntico ao do relatório 002; Croqui: Spools divididos nas juntas 13, 11 e 09</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="n">
+        <v>67</v>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>036</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>Relatório Dimensional</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="n">
+        <v>46259</v>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>I-IS-025-421-510-46-9138</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>002</t>
+        </is>
+      </c>
+      <c r="G68" s="2" t="inlineStr"/>
+      <c r="H68" s="2" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="I68" s="2" t="inlineStr">
+        <is>
+          <t>422-430.pdf</t>
+        </is>
+      </c>
+      <c r="J68" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="K68" s="4" t="inlineStr">
+        <is>
+          <t>Mesmo desenho dos relatórios 021; TAG não consta no relatório (referência é o isométrico); Croqui idêntico ao do relatório 002; Croqui: Spools divididos nas juntas 13, 11 e 09</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>036</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>Relatório Dimensional</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="n">
+        <v>46259</v>
+      </c>
+      <c r="E69" s="2" t="inlineStr">
+        <is>
+          <t>I-IS-025-421-510-46-9138</t>
+        </is>
+      </c>
+      <c r="F69" s="2" t="inlineStr">
+        <is>
+          <t>003</t>
+        </is>
+      </c>
+      <c r="G69" s="2" t="inlineStr"/>
+      <c r="H69" s="2" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="I69" s="2" t="inlineStr">
+        <is>
+          <t>422-430.pdf</t>
+        </is>
+      </c>
+      <c r="J69" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="K69" s="4" t="inlineStr">
+        <is>
+          <t>Mesmo desenho dos relatórios 021; TAG não consta no relatório (referência é o isométrico); Croqui idêntico ao do relatório 002; Croqui: Spools divididos nas juntas 13, 11 e 09</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="n">
+        <v>69</v>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>036</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>Relatório Dimensional</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="n">
+        <v>46259</v>
+      </c>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t>I-IS-025-421-510-46-9138</t>
+        </is>
+      </c>
+      <c r="F70" s="2" t="inlineStr">
+        <is>
+          <t>004</t>
+        </is>
+      </c>
+      <c r="G70" s="2" t="inlineStr"/>
+      <c r="H70" s="2" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="I70" s="2" t="inlineStr">
+        <is>
+          <t>422-430.pdf</t>
+        </is>
+      </c>
+      <c r="J70" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="K70" s="4" t="inlineStr">
+        <is>
+          <t>Mesmo desenho dos relatórios 021; TAG não consta no relatório (referência é o isométrico); Croqui idêntico ao do relatório 002; Croqui: Spools divididos nas juntas 13, 11 e 09</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J44"/>
+  <autoFilter ref="A1:K70"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2461,7 +3928,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J28"/>
+  <dimension ref="A1:K37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -2472,8 +3939,9 @@
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="8" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="70" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="70" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2519,10 +3987,15 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Página no databook</t>
+          <t>Arquivo PDF</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Página no PDF</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Observação</t>
         </is>
@@ -2565,10 +4038,15 @@
           <t>Aprovado</t>
         </is>
       </c>
-      <c r="I2" s="2" t="n">
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>395-421.pdf</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="J2" s="4" t="inlineStr">
+      <c r="K2" s="4" t="inlineStr">
         <is>
           <t>Croqui: Divisão entre spools na junta 8; juntas 4 e 15 solda de campo; spool 02 com sobremetal</t>
         </is>
@@ -2611,10 +4089,15 @@
           <t>Aprovado</t>
         </is>
       </c>
-      <c r="I3" s="2" t="n">
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>395-421.pdf</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="J3" s="4" t="inlineStr">
+      <c r="K3" s="4" t="inlineStr">
         <is>
           <t>Croqui: Spools divididos nas juntas 13, 11 e 09</t>
         </is>
@@ -2653,10 +4136,15 @@
           <t>Aprovado</t>
         </is>
       </c>
-      <c r="I4" s="2" t="n">
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>395-421.pdf</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="J4" s="4" t="inlineStr">
+      <c r="K4" s="4" t="inlineStr">
         <is>
           <t>TAG não consta no relatório (referência é o isométrico)</t>
         </is>
@@ -2699,10 +4187,15 @@
           <t>Aprovado</t>
         </is>
       </c>
-      <c r="I5" s="2" t="n">
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>395-421.pdf</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="J5" s="4" t="inlineStr">
+      <c r="K5" s="4" t="inlineStr">
         <is>
           <t>Prefixo de módulo MO7 removido; Spool não identificado no croqui – considerado spool único 001</t>
         </is>
@@ -2745,10 +4238,15 @@
           <t>Aprovado</t>
         </is>
       </c>
-      <c r="I6" s="2" t="n">
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>395-421.pdf</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="J6" s="4" t="inlineStr">
+      <c r="K6" s="4" t="inlineStr">
         <is>
           <t>Croqui: Extremidades com sobremetal</t>
         </is>
@@ -2791,10 +4289,15 @@
           <t>Aprovado</t>
         </is>
       </c>
-      <c r="I7" s="2" t="n">
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>395-421.pdf</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="J7" s="4" t="inlineStr">
+      <c r="K7" s="4" t="inlineStr">
         <is>
           <t>Croqui: Spool dividido na junta 19; extremidade 01 com sobremetal</t>
         </is>
@@ -2837,10 +4340,15 @@
           <t>Aprovado</t>
         </is>
       </c>
-      <c r="I8" s="2" t="n">
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>395-421.pdf</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="J8" s="4" t="inlineStr">
+      <c r="K8" s="4" t="inlineStr">
         <is>
           <t>Spool não identificado no croqui – considerado spool único 001; Croqui: Extremidade com sobremetal</t>
         </is>
@@ -2883,10 +4391,15 @@
           <t>Aprovado</t>
         </is>
       </c>
-      <c r="I9" s="2" t="n">
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>395-421.pdf</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="J9" s="4" t="inlineStr">
+      <c r="K9" s="4" t="inlineStr">
         <is>
           <t>Spool não identificado no croqui – considerado spool único 001</t>
         </is>
@@ -2929,10 +4442,15 @@
           <t>Aprovado</t>
         </is>
       </c>
-      <c r="I10" s="2" t="n">
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>395-421.pdf</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="J10" s="4" t="inlineStr">
+      <c r="K10" s="4" t="inlineStr">
         <is>
           <t>Croqui: Spool dividido na junta 4</t>
         </is>
@@ -2971,10 +4489,15 @@
           <t>Aprovado</t>
         </is>
       </c>
-      <c r="I11" s="2" t="n">
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>395-421.pdf</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="J11" s="4" t="inlineStr">
+      <c r="K11" s="4" t="inlineStr">
         <is>
           <t>TAG não consta no relatório (referência é o isométrico)</t>
         </is>
@@ -3017,10 +4540,15 @@
           <t>Aprovado</t>
         </is>
       </c>
-      <c r="I12" s="2" t="n">
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>395-421.pdf</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="J12" s="4" t="inlineStr">
+      <c r="K12" s="4" t="inlineStr">
         <is>
           <t>Croqui: Spool dividido na junta 8</t>
         </is>
@@ -3063,10 +4591,15 @@
           <t>Aprovado</t>
         </is>
       </c>
-      <c r="I13" s="2" t="n">
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>395-421.pdf</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="J13" s="4" t="inlineStr">
+      <c r="K13" s="4" t="inlineStr">
         <is>
           <t>Prefixo de módulo MO8 removido; Spool não identificado no croqui – considerado spool único 001</t>
         </is>
@@ -3109,10 +4642,15 @@
           <t>Aprovado</t>
         </is>
       </c>
-      <c r="I14" s="2" t="n">
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>395-421.pdf</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="J14" s="4" t="inlineStr">
+      <c r="K14" s="4" t="inlineStr">
         <is>
           <t>Prefixo de módulo MO5 removido; Spool não identificado no croqui – considerado spool único 001</t>
         </is>
@@ -3151,10 +4689,15 @@
           <t>Aprovado</t>
         </is>
       </c>
-      <c r="I15" s="2" t="n">
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>395-421.pdf</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="J15" s="4" t="inlineStr">
+      <c r="K15" s="4" t="inlineStr">
         <is>
           <t>TAG não consta no relatório (referência é o isométrico); Spool não identificado no croqui – considerado spool único 001; Croqui: Extremidades FT (solda de campo)</t>
         </is>
@@ -3193,10 +4736,15 @@
           <t>Aprovado</t>
         </is>
       </c>
-      <c r="I16" s="2" t="n">
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>395-421.pdf</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="J16" s="4" t="inlineStr">
+      <c r="K16" s="4" t="inlineStr">
         <is>
           <t>TAG não consta no relatório (referência é o isométrico); Spool não identificado no croqui – considerado spool único 001; Croqui: Extremidade FT (solda de campo)</t>
         </is>
@@ -3235,10 +4783,15 @@
           <t>Aprovado</t>
         </is>
       </c>
-      <c r="I17" s="2" t="n">
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>395-421.pdf</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="n">
         <v>16</v>
       </c>
-      <c r="J17" s="4" t="inlineStr">
+      <c r="K17" s="4" t="inlineStr">
         <is>
           <t>TAG não consta no relatório (referência é o isométrico); Spool não identificado no croqui – considerado spool único 001; Croqui idêntico ao do relatório 007; Croqui: Extremidade com sobremetal</t>
         </is>
@@ -3277,10 +4830,15 @@
           <t>Aprovado</t>
         </is>
       </c>
-      <c r="I18" s="2" t="n">
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>395-421.pdf</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="J18" s="4" t="inlineStr">
+      <c r="K18" s="4" t="inlineStr">
         <is>
           <t>TAG não consta no relatório (referência é o isométrico); Croqui idêntico ao do relatório 005; Croqui: Extremidades com sobremetal</t>
         </is>
@@ -3319,10 +4877,15 @@
           <t>Aprovado</t>
         </is>
       </c>
-      <c r="I19" s="2" t="n">
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>395-421.pdf</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="J19" s="4" t="inlineStr">
+      <c r="K19" s="4" t="inlineStr">
         <is>
           <t>TAG não consta no relatório (referência é o isométrico)</t>
         </is>
@@ -3361,10 +4924,15 @@
           <t>Aprovado</t>
         </is>
       </c>
-      <c r="I20" s="2" t="n">
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>395-421.pdf</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="n">
         <v>19</v>
       </c>
-      <c r="J20" s="4" t="inlineStr">
+      <c r="K20" s="4" t="inlineStr">
         <is>
           <t>TAG não consta no relatório (referência é o isométrico); Spool não identificado no croqui – considerado spool único 001; Croqui idêntico ao do relatório 008</t>
         </is>
@@ -3403,10 +4971,15 @@
           <t>Aprovado</t>
         </is>
       </c>
-      <c r="I21" s="2" t="n">
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>395-421.pdf</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="J21" s="4" t="inlineStr">
+      <c r="K21" s="4" t="inlineStr">
         <is>
           <t>TAG não consta no relatório (referência é o isométrico); Croqui idêntico ao do relatório 009; Croqui: Spool dividido na junta 4</t>
         </is>
@@ -3445,12 +5018,17 @@
           <t>Aprovado</t>
         </is>
       </c>
-      <c r="I22" s="2" t="n">
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>395-421.pdf</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="n">
         <v>21</v>
       </c>
-      <c r="J22" s="4" t="inlineStr">
-        <is>
-          <t>TAG não consta no relatório (referência é o isométrico); Croqui idêntico ao do relatório 002; Croqui: Spools divididos nas juntas 13, 11 e 09</t>
+      <c r="K22" s="4" t="inlineStr">
+        <is>
+          <t>Mesmo desenho dos relatórios 036; TAG não consta no relatório (referência é o isométrico); Croqui idêntico ao do relatório 002; Croqui: Spools divididos nas juntas 13, 11 e 09</t>
         </is>
       </c>
     </row>
@@ -3491,10 +5069,15 @@
           <t>Aprovado</t>
         </is>
       </c>
-      <c r="I23" s="2" t="n">
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>395-421.pdf</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="n">
         <v>22</v>
       </c>
-      <c r="J23" s="4" t="inlineStr">
+      <c r="K23" s="4" t="inlineStr">
         <is>
           <t>Prefixo de módulo MO7 removido; Spool não identificado no croqui – considerado spool único 001</t>
         </is>
@@ -3537,10 +5120,15 @@
           <t>Aprovado</t>
         </is>
       </c>
-      <c r="I24" s="2" t="n">
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>395-421.pdf</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="n">
         <v>23</v>
       </c>
-      <c r="J24" s="4" t="inlineStr">
+      <c r="K24" s="4" t="inlineStr">
         <is>
           <t>Prefixo de módulo MO6 removido</t>
         </is>
@@ -3583,10 +5171,15 @@
           <t>Aprovado</t>
         </is>
       </c>
-      <c r="I25" s="2" t="n">
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>395-421.pdf</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="n">
         <v>24</v>
       </c>
-      <c r="J25" s="4" t="inlineStr">
+      <c r="K25" s="4" t="inlineStr">
         <is>
           <t>Prefixo de módulo MO7 removido; Croqui: Spool dividido nas juntas 06 e 20</t>
         </is>
@@ -3629,10 +5222,15 @@
           <t>Aprovado</t>
         </is>
       </c>
-      <c r="I26" s="2" t="n">
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>395-421.pdf</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="n">
         <v>25</v>
       </c>
-      <c r="J26" s="4" t="inlineStr">
+      <c r="K26" s="4" t="inlineStr">
         <is>
           <t>Prefixo de módulo MO5 removido</t>
         </is>
@@ -3675,10 +5273,15 @@
           <t>Aprovado</t>
         </is>
       </c>
-      <c r="I27" s="2" t="n">
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>395-421.pdf</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="n">
         <v>26</v>
       </c>
-      <c r="J27" s="4" t="inlineStr">
+      <c r="K27" s="4" t="inlineStr">
         <is>
           <t>Prefixo de módulo MO8 removido; Croqui: Spool dividido nas juntas 04 e 12</t>
         </is>
@@ -3721,17 +5324,453 @@
           <t>Aprovado</t>
         </is>
       </c>
-      <c r="I28" s="2" t="n">
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>395-421.pdf</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="n">
         <v>27</v>
       </c>
-      <c r="J28" s="4" t="inlineStr">
+      <c r="K28" s="4" t="inlineStr">
         <is>
           <t>Prefixo de módulo MO5 removido; Croqui: Spool dividido na junta 04</t>
         </is>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>028</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Relatório Dimensional</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="n">
+        <v>46265</v>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>I-IS-025-421-510-46-9067</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr"/>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>001, 002, 003</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>422-430.pdf</t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K29" s="4" t="inlineStr">
+        <is>
+          <t>TAG não consta no relatório (referência é o isométrico); Croqui: Spools divididos nas juntas 04 e 05; extremidades FT</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>029</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Relatório Dimensional</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="n">
+        <v>46260</v>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>I-IS-025-421-510-46-9141</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr"/>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>001, 002</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>422-430.pdf</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K30" s="4" t="inlineStr">
+        <is>
+          <t>TAG não consta no relatório (referência é o isométrico); Croqui idêntico ao do relatório 006; Croqui: Spool dividido na junta 19; extremidade 01 com sobremetal</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>030</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Relatório Dimensional</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="n">
+        <v>46266</v>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>MO8-6´´-B3B-MR-5407B-PP-2 FL 2/2</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>6"-B3B-MR-5407B</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>001, 002, 003, 004</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>422-430.pdf</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="K31" s="4" t="inlineStr">
+        <is>
+          <t>Prefixo de módulo MO8 removido; Croqui: Spool dividido nas juntas 08, 16 e 28</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>031</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Relatório Dimensional</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="n">
+        <v>46265</v>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>I-IS-025-421-510-46-9048</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr"/>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>001, 002, 003</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>422-430.pdf</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="K32" s="4" t="inlineStr">
+        <is>
+          <t>TAG não consta no relatório (referência é o isométrico); Croqui: Spools divididos nas juntas 08 e 09; extremidades FT</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>032</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>Relatório Dimensional</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="n">
+        <v>46265</v>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>I-IS-025-421-510-46-9049</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr"/>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>001, 002, 003</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>422-430.pdf</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="K33" s="4" t="inlineStr">
+        <is>
+          <t>TAG não consta no relatório (referência é o isométrico); Croqui: Spools divididos nas juntas 24 e 25; extremidades FT</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>033</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Relatório Dimensional</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="n">
+        <v>46266</v>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>6´´-B3B-MR-5407A-PP-2</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>6"-B3B-MR-5407A</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>002, 003</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>422-430.pdf</t>
+        </is>
+      </c>
+      <c r="J34" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="K34" s="4" t="inlineStr">
+        <is>
+          <t>Croqui: Spool dividido nas juntas 08 e 12</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>034</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Relatório Dimensional</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="n">
+        <v>46259</v>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>I-IS-025-421-510-46-9137</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr"/>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>001, 002</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t>422-430.pdf</t>
+        </is>
+      </c>
+      <c r="J35" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="K35" s="4" t="inlineStr">
+        <is>
+          <t>TAG não consta no relatório (referência é o isométrico); Croqui idêntico ao do relatório 001; Croqui: Spool dividido na junta 8; juntas 4 e 15 FW</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>035</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>Relatório Dimensional</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="n">
+        <v>46265</v>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>I-IS-025-421-510-46-9066</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr"/>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>001, 002, 003</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>422-430.pdf</t>
+        </is>
+      </c>
+      <c r="J36" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="K36" s="4" t="inlineStr">
+        <is>
+          <t>TAG não consta no relatório (referência é o isométrico); Croqui: Spools divididos nas juntas 16 e 17; extremidades FT</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>036</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>Relatório Dimensional</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="n">
+        <v>46259</v>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>I-IS-025-421-510-46-9138</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr"/>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>001, 002, 003, 004</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>422-430.pdf</t>
+        </is>
+      </c>
+      <c r="J37" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="K37" s="4" t="inlineStr">
+        <is>
+          <t>Mesmo desenho dos relatórios 021; TAG não consta no relatório (referência é o isométrico); Croqui idêntico ao do relatório 002; Croqui: Spools divididos nas juntas 13, 11 e 09</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J28"/>
+  <autoFilter ref="A1:K37"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>